<commit_message>
Try to make a good sextupole correction
</commit_message>
<xml_diff>
--- a/MADX/tbl/Distortion.xlsx
+++ b/MADX/tbl/Distortion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Bell 1/GIT_REPOS/NICA/MADX/tbl/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B0C1447C-BF1E-604E-AA31-FF70967EE643}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96CB795E-DBDE-6E49-B793-0BED5CBCB1F8}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="10000" windowHeight="18000" xr2:uid="{390887FB-72E9-3345-97DB-AFEA83EA7214}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="265">
   <si>
     <t>MUX</t>
   </si>
@@ -736,6 +736,90 @@
   </si>
   <si>
     <t>9.425710399</t>
+  </si>
+  <si>
+    <t>9.434324704</t>
+  </si>
+  <si>
+    <t>9.425235136</t>
+  </si>
+  <si>
+    <t>9.437194837</t>
+  </si>
+  <si>
+    <t>9.436652349</t>
+  </si>
+  <si>
+    <t>9.446102245</t>
+  </si>
+  <si>
+    <t>9.44935452</t>
+  </si>
+  <si>
+    <t>9.460689444</t>
+  </si>
+  <si>
+    <t>9.464089343</t>
+  </si>
+  <si>
+    <t>9.480406394</t>
+  </si>
+  <si>
+    <t>9.480314651</t>
+  </si>
+  <si>
+    <t>9.505304272</t>
+  </si>
+  <si>
+    <t>9.495010459</t>
+  </si>
+  <si>
+    <t>9.53915132</t>
+  </si>
+  <si>
+    <t>9.504132808</t>
+  </si>
+  <si>
+    <t>9.612115892</t>
+  </si>
+  <si>
+    <t>9.506164483</t>
+  </si>
+  <si>
+    <t>9.437432525</t>
+  </si>
+  <si>
+    <t>9.414220361</t>
+  </si>
+  <si>
+    <t>9.445993519</t>
+  </si>
+  <si>
+    <t>9.403046714</t>
+  </si>
+  <si>
+    <t>9.459119766</t>
+  </si>
+  <si>
+    <t>9.391508502</t>
+  </si>
+  <si>
+    <t>9.476096637</t>
+  </si>
+  <si>
+    <t>9.379310188</t>
+  </si>
+  <si>
+    <t>9.498580832</t>
+  </si>
+  <si>
+    <t>9.363931521</t>
+  </si>
+  <si>
+    <t>9.551249488</t>
+  </si>
+  <si>
+    <t>9.331331033</t>
   </si>
 </sst>
 </file>
@@ -1096,7 +1180,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E125C895-7F94-C544-9EAF-D55C3C631C56}">
-  <dimension ref="A1:G94"/>
+  <dimension ref="A1:G118"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="4" width="14.1640625" customWidth="1"/>
@@ -2345,16 +2429,242 @@
       <c r="B90" s="1"/>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B91" s="1"/>
+      <c r="A91">
+        <v>4</v>
+      </c>
+      <c r="B91" t="s">
+        <v>10</v>
+      </c>
+      <c r="C91" t="s">
+        <v>237</v>
+      </c>
+      <c r="D91" t="s">
+        <v>238</v>
+      </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B92" s="1"/>
+      <c r="A92">
+        <v>4</v>
+      </c>
+      <c r="B92" t="s">
+        <v>9</v>
+      </c>
+      <c r="C92" t="s">
+        <v>239</v>
+      </c>
+      <c r="D92" t="s">
+        <v>240</v>
+      </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B93" s="1"/>
+      <c r="A93">
+        <v>4</v>
+      </c>
+      <c r="B93" t="s">
+        <v>15</v>
+      </c>
+      <c r="C93" t="s">
+        <v>241</v>
+      </c>
+      <c r="D93" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B94" s="1"/>
+      <c r="A94">
+        <v>4</v>
+      </c>
+      <c r="B94" t="s">
+        <v>18</v>
+      </c>
+      <c r="C94" t="s">
+        <v>243</v>
+      </c>
+      <c r="D94" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A95">
+        <v>4</v>
+      </c>
+      <c r="B95" t="s">
+        <v>27</v>
+      </c>
+      <c r="C95" t="s">
+        <v>245</v>
+      </c>
+      <c r="D95" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A96">
+        <v>4</v>
+      </c>
+      <c r="B96" t="s">
+        <v>32</v>
+      </c>
+      <c r="C96" t="s">
+        <v>247</v>
+      </c>
+      <c r="D96" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A97">
+        <v>4</v>
+      </c>
+      <c r="B97" t="s">
+        <v>39</v>
+      </c>
+      <c r="C97" t="s">
+        <v>249</v>
+      </c>
+      <c r="D97" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A98">
+        <v>4</v>
+      </c>
+      <c r="B98" t="s">
+        <v>44</v>
+      </c>
+      <c r="C98" t="s">
+        <v>251</v>
+      </c>
+      <c r="D98" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A99">
+        <v>4</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C99" t="s">
+        <v>253</v>
+      </c>
+      <c r="D99" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A100">
+        <v>4</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C100" t="s">
+        <v>255</v>
+      </c>
+      <c r="D100" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A101">
+        <v>4</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C101" t="s">
+        <v>257</v>
+      </c>
+      <c r="D101" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A102">
+        <v>4</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C102" t="s">
+        <v>259</v>
+      </c>
+      <c r="D102" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A103">
+        <v>4</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C103" t="s">
+        <v>261</v>
+      </c>
+      <c r="D103" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A104">
+        <v>4</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="D104" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B105" s="1"/>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B106" s="1"/>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B107" s="1"/>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B108" s="1"/>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B109" s="1"/>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B110" s="1"/>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B111" s="1"/>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B112" s="1"/>
+    </row>
+    <row r="113" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B113" s="1"/>
+    </row>
+    <row r="114" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B114" s="1"/>
+    </row>
+    <row r="115" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B115" s="1"/>
+    </row>
+    <row r="116" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B116" s="1"/>
+    </row>
+    <row r="117" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B117" s="1"/>
+    </row>
+    <row r="118" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B118" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>